<commit_message>
Updated with Loves Data
</commit_message>
<xml_diff>
--- a/analysis/data/FP_FN_ALL_2026-01-11_Ava.xlsx
+++ b/analysis/data/FP_FN_ALL_2026-01-11_Ava.xlsx
@@ -1,9 +1,9 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29819"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29825"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{9B99D5C0-FB73-4834-B38A-A9AD8D970C34}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{D1677F28-54FD-414B-94ED-60739FF399E8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="740" windowWidth="29400" windowHeight="18380" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>

</xml_diff>